<commit_message>
Value alone in every cell; units and uncertainty out
The register is a results overview and document reference, so a cell holds the
bare result and nothing else. "26.14 %w/w (U 1.61)" becomes 26.14; "<2 ug/kg"
becomes <2; "10.3% (U +-0.2) [flag...]" becomes 10.3 with the flag carried by
the cell colour. Units move to the column headers (Aflatoxins ug/kg, Pb mg/kg,
TAMC CFU/g); expanded measurement uncertainty leaves the table - it remains in
Full Data verbatim. Notations that are the result itself - <LOQ, BLQ, ND,
Odgovara, <10^2 and >10 - are untouched, and severity is judged on the original
text so no flag is lost by the cleaning.

Applied to the one-sheet Batch Release QC Register and the THC-by-strain table;
both keep per-row CoA code, date of issue and issuing institution.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyBhj47i7bhaCyNMB1iwdv
</commit_message>
<xml_diff>
--- a/ingestion/coa_track/letta-imb-coas/exports/PP_THC_by_Strain.xlsx
+++ b/ingestion/coa_track/letta-imb-coas/exports/PP_THC_by_Strain.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Total Δ⁹-THC</t>
+          <t>Total Δ⁹-THC % w/w</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -634,7 +634,7 @@
       <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>21.80%</t>
+          <t>21.80</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -669,7 +669,7 @@
       <c r="C7" s="12" t="n"/>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>26.14 %w/w (U 1.61)</t>
+          <t>26.14</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -717,7 +717,7 @@
       <c r="C9" s="18" t="inlineStr"/>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>21.03%</t>
+          <t>21.03</t>
         </is>
       </c>
       <c r="E9" s="21" t="inlineStr">
@@ -749,7 +749,7 @@
     <row r="10">
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>25.01 %w/w (U 1.54)</t>
+          <t>25.01</t>
         </is>
       </c>
       <c r="E10" s="21" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="D11" s="20" t="inlineStr">
         <is>
-          <t>23.42%</t>
+          <t>23.42</t>
         </is>
       </c>
       <c r="E11" s="21" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="D12" s="28" t="inlineStr">
         <is>
-          <t>20.39%</t>
+          <t>20.39</t>
         </is>
       </c>
       <c r="E12" s="29" t="inlineStr">
@@ -887,7 +887,7 @@
       <c r="C14" s="9" t="inlineStr"/>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>23.00%</t>
+          <t>23.00</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>20.29%</t>
+          <t>20.29</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -964,7 +964,7 @@
     <row r="16">
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>24.05 %w/w (U 1.48)</t>
+          <t>24.05</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>14.93%</t>
+          <t>14.93</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>23.70%</t>
+          <t>23.70</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D20" s="20" t="inlineStr">
         <is>
-          <t>17.22%</t>
+          <t>17.22</t>
         </is>
       </c>
       <c r="E20" s="21" t="inlineStr">
@@ -1138,7 +1138,7 @@
     <row r="21">
       <c r="D21" s="20" t="inlineStr">
         <is>
-          <t>18.67 %w/w (U 1.15)</t>
+          <t>18.67</t>
         </is>
       </c>
       <c r="E21" s="21" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>15.95%</t>
+          <t>15.95</t>
         </is>
       </c>
       <c r="E22" s="21" t="inlineStr">
@@ -1224,7 +1224,7 @@
       <c r="C23" s="22" t="inlineStr"/>
       <c r="D23" s="20" t="inlineStr">
         <is>
-          <t>15.35%</t>
+          <t>15.35</t>
         </is>
       </c>
       <c r="E23" s="21" t="inlineStr"/>
@@ -1261,7 +1261,7 @@
       <c r="C24" s="26" t="inlineStr"/>
       <c r="D24" s="28" t="inlineStr">
         <is>
-          <t>17.94%</t>
+          <t>17.94</t>
         </is>
       </c>
       <c r="E24" s="29" t="inlineStr"/>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>20.79%</t>
+          <t>20.79</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>23.19%</t>
+          <t>23.19</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -1386,7 +1386,7 @@
     <row r="28">
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>22.61 %w/w (U 1.39)</t>
+          <t>22.61</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>25.45%</t>
+          <t>25.45</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>18.98%</t>
+          <t>18.98</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -1508,7 +1508,7 @@
     <row r="31">
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>18.52 %w/w (U 1.14)</t>
+          <t>18.52</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>24.89%</t>
+          <t>24.89</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>21.36%</t>
+          <t>21.36</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>19.81%</t>
+          <t>19.81</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>21.29%</t>
+          <t>21.29</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>14.83%</t>
+          <t>14.83</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
@@ -1765,7 +1765,7 @@
     <row r="37">
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>15.70% w/w (U 0.96% w/w)</t>
+          <t>15.70</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>25.73%</t>
+          <t>25.73</t>
         </is>
       </c>
       <c r="E38" s="14" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="D40" s="20" t="inlineStr">
         <is>
-          <t>18.67%</t>
+          <t>18.67</t>
         </is>
       </c>
       <c r="E40" s="21" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="D41" s="28" t="inlineStr">
         <is>
-          <t>16.82%</t>
+          <t>16.82</t>
         </is>
       </c>
       <c r="E41" s="29" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>15.38%</t>
+          <t>15.38</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>18.27%</t>
+          <t>18.27</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
@@ -2036,7 +2036,7 @@
     <row r="45">
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>18.04 %w/w (U 1.11)</t>
+          <t>18.04</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>16.55%</t>
+          <t>16.55</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>14.16%</t>
+          <t>14.16</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>9.43%</t>
+          <t>9.43</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
@@ -2212,7 +2212,7 @@
       <c r="C49" s="9" t="inlineStr"/>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>8.00%</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
@@ -2253,7 +2253,7 @@
       <c r="C50" s="15" t="inlineStr"/>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>8.09 %w/w (U ±0.50)</t>
+          <t>8.09</t>
         </is>
       </c>
       <c r="E50" s="14" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="D52" s="20" t="inlineStr">
         <is>
-          <t>22.43%</t>
+          <t>22.43</t>
         </is>
       </c>
       <c r="E52" s="21" t="inlineStr">
@@ -2337,7 +2337,7 @@
     <row r="53">
       <c r="D53" s="20" t="inlineStr">
         <is>
-          <t>21.61 %w/w (U 1.33)</t>
+          <t>21.61</t>
         </is>
       </c>
       <c r="E53" s="21" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="D54" s="28" t="inlineStr">
         <is>
-          <t>20.39%</t>
+          <t>20.39</t>
         </is>
       </c>
       <c r="E54" s="29" t="inlineStr">
@@ -2434,7 +2434,7 @@
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>16.56%</t>
+          <t>16.56</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -2466,7 +2466,7 @@
     <row r="57">
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>18.91% w/w (U 1.16% w/w)</t>
+          <t>18.91</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="D58" s="13" t="inlineStr">
         <is>
-          <t>21.51%</t>
+          <t>21.51</t>
         </is>
       </c>
       <c r="E58" s="14" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="D60" s="20" t="inlineStr">
         <is>
-          <t>22.11%</t>
+          <t>22.11</t>
         </is>
       </c>
       <c r="E60" s="21" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="D61" s="28" t="inlineStr">
         <is>
-          <t>21.67%</t>
+          <t>21.67</t>
         </is>
       </c>
       <c r="E61" s="29" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>10.01%</t>
+          <t>10.01</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
@@ -2705,7 +2705,7 @@
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>14.06%</t>
+          <t>14.06</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
@@ -2737,7 +2737,7 @@
     <row r="65">
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>12.25% w/w (U 0.75% w/w)</t>
+          <t>12.25</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -2778,7 +2778,7 @@
       <c r="C66" s="15" t="inlineStr"/>
       <c r="D66" s="13" t="inlineStr">
         <is>
-          <t>13.33%</t>
+          <t>13.33</t>
         </is>
       </c>
       <c r="E66" s="14" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="D68" s="28" t="inlineStr">
         <is>
-          <t>8.02%</t>
+          <t>8.02</t>
         </is>
       </c>
       <c r="E68" s="29" t="inlineStr">
@@ -2882,7 +2882,7 @@
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>24.96%</t>
+          <t>24.96</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>20.84%</t>
+          <t>20.84</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
@@ -2959,7 +2959,7 @@
     <row r="72">
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>18.29% w/w (U 1.12% w/w)</t>
+          <t>18.29</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="D73" s="13" t="inlineStr">
         <is>
-          <t>22.30%</t>
+          <t>22.30</t>
         </is>
       </c>
       <c r="E73" s="14" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="D75" s="28" t="inlineStr">
         <is>
-          <t>16.93%</t>
+          <t>16.93</t>
         </is>
       </c>
       <c r="E75" s="29" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>10.96%</t>
+          <t>10.96</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
@@ -3149,7 +3149,7 @@
       <c r="C78" s="9" t="inlineStr"/>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>11.20 %w/w (U ±0.69)</t>
+          <t>11.20</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
@@ -3190,7 +3190,7 @@
       <c r="C79" s="15" t="inlineStr"/>
       <c r="D79" s="13" t="inlineStr">
         <is>
-          <t>9.20 %w/w (U ±0.57)</t>
+          <t>9.20</t>
         </is>
       </c>
       <c r="E79" s="14" t="inlineStr">
@@ -3238,7 +3238,7 @@
       <c r="C81" s="26" t="inlineStr"/>
       <c r="D81" s="28" t="inlineStr">
         <is>
-          <t>11.53 %w/w (U ±0.71)</t>
+          <t>11.53</t>
         </is>
       </c>
       <c r="E81" s="29" t="inlineStr">
@@ -3286,7 +3286,7 @@
       <c r="C83" s="9" t="inlineStr"/>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>19.14 %w/w (U ±1.18)</t>
+          <t>19.14</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
@@ -3327,7 +3327,7 @@
       <c r="C84" s="5" t="inlineStr"/>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>25.27 %w/w (U ±1.55)</t>
+          <t>25.27</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr">
@@ -3359,7 +3359,7 @@
     <row r="85">
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>20.21 %w/w (U ±1.24)</t>
+          <t>20.21</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
@@ -3400,7 +3400,7 @@
       <c r="C86" s="5" t="inlineStr"/>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>19.84 %w/w (U ±1.22)</t>
+          <t>19.84</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
@@ -3435,7 +3435,7 @@
       <c r="C87" s="12" t="n"/>
       <c r="D87" s="13" t="inlineStr">
         <is>
-          <t>21.84 %w/w (U ±1.34)</t>
+          <t>21.84</t>
         </is>
       </c>
       <c r="E87" s="14" t="inlineStr">
@@ -3483,7 +3483,7 @@
       <c r="C89" s="26" t="inlineStr"/>
       <c r="D89" s="28" t="inlineStr">
         <is>
-          <t>17.04 %w/w (U ±1.05)</t>
+          <t>17.04</t>
         </is>
       </c>
       <c r="E89" s="29" t="inlineStr">
@@ -3531,7 +3531,7 @@
       <c r="C91" s="15" t="inlineStr"/>
       <c r="D91" s="13" t="inlineStr">
         <is>
-          <t>13.35%</t>
+          <t>13.35</t>
         </is>
       </c>
       <c r="E91" s="14" t="inlineStr"/>
@@ -3575,7 +3575,7 @@
       <c r="C93" s="22" t="inlineStr"/>
       <c r="D93" s="20" t="inlineStr">
         <is>
-          <t>14.68%</t>
+          <t>14.68</t>
         </is>
       </c>
       <c r="E93" s="21" t="inlineStr"/>
@@ -3612,7 +3612,7 @@
       <c r="C94" s="22" t="inlineStr"/>
       <c r="D94" s="20" t="inlineStr">
         <is>
-          <t>16.69%</t>
+          <t>16.69</t>
         </is>
       </c>
       <c r="E94" s="21" t="inlineStr"/>
@@ -3649,7 +3649,7 @@
       <c r="C95" s="26" t="inlineStr"/>
       <c r="D95" s="28" t="inlineStr">
         <is>
-          <t>20.83%</t>
+          <t>20.83</t>
         </is>
       </c>
       <c r="E95" s="29" t="inlineStr">
@@ -3697,7 +3697,7 @@
       <c r="C97" s="9" t="inlineStr"/>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>18.16%</t>
+          <t>18.16</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr"/>
@@ -3734,7 +3734,7 @@
       <c r="C98" s="5" t="inlineStr"/>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>19.64%</t>
+          <t>19.64</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr"/>
@@ -3765,7 +3765,7 @@
       <c r="C99" s="12" t="n"/>
       <c r="D99" s="13" t="inlineStr">
         <is>
-          <t>13.93%</t>
+          <t>13.93</t>
         </is>
       </c>
       <c r="E99" s="14" t="inlineStr"/>
@@ -3809,7 +3809,7 @@
       <c r="C101" s="22" t="inlineStr"/>
       <c r="D101" s="20" t="inlineStr">
         <is>
-          <t>17.13%</t>
+          <t>17.13</t>
         </is>
       </c>
       <c r="E101" s="21" t="inlineStr"/>
@@ -3846,7 +3846,7 @@
       <c r="C102" s="22" t="inlineStr"/>
       <c r="D102" s="20" t="inlineStr">
         <is>
-          <t>21.92%</t>
+          <t>21.92</t>
         </is>
       </c>
       <c r="E102" s="21" t="inlineStr">
@@ -3891,7 +3891,7 @@
       </c>
       <c r="D103" s="28" t="inlineStr">
         <is>
-          <t>17.84 %w/w (U 1.10 %w/w, k=2)</t>
+          <t>17.84</t>
         </is>
       </c>
       <c r="E103" s="29" t="inlineStr">
@@ -3939,7 +3939,7 @@
       <c r="C105" s="9" t="inlineStr"/>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>18.29%</t>
+          <t>18.29</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -3980,7 +3980,7 @@
       <c r="C106" s="9" t="inlineStr"/>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>12.39%</t>
+          <t>12.39</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="D107" s="13" t="inlineStr">
         <is>
-          <t>18.86 %w/w (U 1.16 %w/w, k=2)</t>
+          <t>18.86</t>
         </is>
       </c>
       <c r="E107" s="14" t="inlineStr">
@@ -4073,7 +4073,7 @@
       <c r="C109" s="22" t="inlineStr"/>
       <c r="D109" s="20" t="inlineStr">
         <is>
-          <t>17.59%</t>
+          <t>17.59</t>
         </is>
       </c>
       <c r="E109" s="21" t="inlineStr">
@@ -4114,7 +4114,7 @@
       <c r="C110" s="22" t="inlineStr"/>
       <c r="D110" s="20" t="inlineStr">
         <is>
-          <t>18.98%</t>
+          <t>18.98</t>
         </is>
       </c>
       <c r="E110" s="21" t="inlineStr">
@@ -4159,7 +4159,7 @@
       </c>
       <c r="D111" s="28" t="inlineStr">
         <is>
-          <t>16.70 %w/w (U 1.03 %w/w, k=2)</t>
+          <t>16.70</t>
         </is>
       </c>
       <c r="E111" s="29" t="inlineStr">
@@ -4207,7 +4207,7 @@
       <c r="C113" s="9" t="inlineStr"/>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>20.54%</t>
+          <t>20.54</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -4248,7 +4248,7 @@
       <c r="C114" s="9" t="inlineStr"/>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>15.16%</t>
+          <t>15.16</t>
         </is>
       </c>
       <c r="E114" s="8" t="inlineStr">
@@ -4289,7 +4289,7 @@
       <c r="C115" s="9" t="inlineStr"/>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>18.58%</t>
+          <t>18.58</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
@@ -4334,7 +4334,7 @@
       </c>
       <c r="D116" s="13" t="inlineStr">
         <is>
-          <t>20.32 %w/w (U 1.25 %w/w, k=2)</t>
+          <t>20.32</t>
         </is>
       </c>
       <c r="E116" s="14" t="inlineStr">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="D118" s="20" t="inlineStr">
         <is>
-          <t>26.32%</t>
+          <t>26.32</t>
         </is>
       </c>
       <c r="E118" s="21" t="inlineStr">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="D119" s="20" t="inlineStr">
         <is>
-          <t>25.72%</t>
+          <t>25.72</t>
         </is>
       </c>
       <c r="E119" s="21" t="inlineStr">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="D120" s="28" t="inlineStr">
         <is>
-          <t>24.78%</t>
+          <t>24.78</t>
         </is>
       </c>
       <c r="E120" s="29" t="inlineStr">
@@ -4528,7 +4528,7 @@
       </c>
       <c r="D122" s="13" t="inlineStr">
         <is>
-          <t>17.32 %w/w (U 1.06 %w/w, k=2)</t>
+          <t>17.32</t>
         </is>
       </c>
       <c r="E122" s="14" t="inlineStr">
@@ -4580,7 +4580,7 @@
       </c>
       <c r="D124" s="20" t="inlineStr">
         <is>
-          <t>7.91 %w/w (U 0.49 %w/w, k=2)</t>
+          <t>7.91</t>
         </is>
       </c>
       <c r="E124" s="21" t="inlineStr">
@@ -4621,7 +4621,7 @@
       <c r="C125" s="18" t="inlineStr"/>
       <c r="D125" s="20" t="inlineStr">
         <is>
-          <t>19.96%</t>
+          <t>19.96</t>
         </is>
       </c>
       <c r="E125" s="21" t="inlineStr">
@@ -4656,7 +4656,7 @@
       <c r="C126" s="12" t="n"/>
       <c r="D126" s="28" t="inlineStr">
         <is>
-          <t>20.03 %w/w (U 1.23 %w/w, k=2)</t>
+          <t>20.03</t>
         </is>
       </c>
       <c r="E126" s="29" t="inlineStr">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="D128" s="13" t="inlineStr">
         <is>
-          <t>17.67 %w/w (U 1.09 %w/w, k=2)</t>
+          <t>17.67</t>
         </is>
       </c>
       <c r="E128" s="14" t="inlineStr">
@@ -4756,7 +4756,7 @@
       <c r="C130" s="18" t="inlineStr"/>
       <c r="D130" s="20" t="inlineStr">
         <is>
-          <t>14.97%</t>
+          <t>14.97</t>
         </is>
       </c>
       <c r="E130" s="21" t="inlineStr">
@@ -4791,7 +4791,7 @@
       <c r="C131" s="12" t="n"/>
       <c r="D131" s="28" t="inlineStr">
         <is>
-          <t>17.31 %w/w (U 1.06 %w/w, k=2)</t>
+          <t>17.31</t>
         </is>
       </c>
       <c r="E131" s="29" t="inlineStr">

</xml_diff>